<commit_message>
Alzey: Techem ausgewertet, CO2-Anteil und Versammlung ergaenzt
Techems eigene Verbrauchsanalyse weist die Wohnung mit 208 Prozent ueber dem
Durchschnittsnutzer aus, 2023 waren es 172 Prozent. 364 kWh je Quadratmeter
gegenueber ueblichen 130 bis 150. Der Wohnzimmer-Heizkoerper macht ueber die
Haelfte des Verbrauchs aus.

Neues Blatt in der Abrechnungsdatei mit den Zahlen, der Raumverteilung und
einer Pruefreihenfolge: Bewertungsfaktoren, Rohrwaerme nach VDI 2077,
Thermostate, Lage im obersten Geschoss.

Nebenbefund CO2-Kostenaufteilungsgesetz: Der Vermieter traegt 30 Prozent,
2024 waren das 43,85 EUR. Techem weist sie aus, zieht sie aber nicht ab -
Zeile dafuer in der Abrechnung ergaenzt.

Dazu die Beschluesse der Versammlung vom 20.07.2026, darunter der neue
Verwaltervertrag ab 2027 mit SEPA- und Portalpflicht.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2Vxc1sWTkdQ9c9u5jSatw
</commit_message>
<xml_diff>
--- a/10_Output/2026-10-26-nebenkosten-2025-alzey-mazineler.xlsx
+++ b/10_Output/2026-10-26-nebenkosten-2025-alzey-mazineler.xlsx
@@ -10,9 +10,11 @@
   <sheets>
     <sheet name="Abrechnung" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Hinweise und Fristen" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Heizkosten pruefen" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Abrechnung!$A$1:$E$46</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Abrechnung!$A$1:$E$47</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">'Heizkosten pruefen'!$A$1:$E$32</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Hinweise und Fristen'!$A$1:$B$22</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -68,12 +70,25 @@
         </r>
       </text>
     </comment>
+    <comment ref="E34" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">FEHLT: Nach dem CO₂-Kostenaufteilungsgesetz trägt der Vermieter einen Teil der CO₂-Abgabe. Techem weist ihn auf der Abrechnung je Bewohner aus, weil die Verwaltung ihn nicht von den Brennstoffkosten abzieht.
+2024 waren es 43,85 €. Den Wert für 2025 aus der Techem-Abrechnung 2025 übernehmen.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="104">
   <si>
     <t xml:space="preserve">Sascha Coldewey</t>
   </si>
@@ -177,6 +192,9 @@
     <t xml:space="preserve">abzüglich Ihrer Vorauszahlungen</t>
   </si>
   <si>
+    <t xml:space="preserve">abzüglich Erstattung CO₂-Kosten (Vermieteranteil 30 %)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ein negatives Ergebnis ist eine Nachzahlung des Mieters, ein positives sein Guthaben.</t>
   </si>
   <si>
@@ -238,15 +256,161 @@
   </si>
   <si>
     <t xml:space="preserve">Die Wartung (4,87 €) ist umlagefähig, die Miete der Geräte (14,36 €) nicht. Die Verwaltung trennt das korrekt — in der Abrechnung steht nur die Wartung.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Heizkosten sind der Knackpunkt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grundlage: Techem-Abrechnung 2024, Nutzer 0144.01.006.01, Lage 2GL. Die Abrechnung 2025 liegt noch nicht vor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Techem sagt es selbst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bewertung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verbrauch der Wohnung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.158 kWh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.360 kWh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">witterungsbereinigt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Durchschnittsnutzer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.549 kWh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.584 kWh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Techems Vergleichsgruppe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abweichung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+208 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+172 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Techems eigene Angabe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verbrauch je Quadratmeter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">364 kWh/qm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">421 kWh/qm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">üblich sind 130 bis 150</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Befund ist über zwei Jahre stabil und stammt nicht von mir, sondern aus Techems eigener Verbrauchsanalyse. Die Wohnung verbraucht dreimal so viel wie vergleichbare Wohnungen. Das erklärt die 3.729,58 € für 2024 — sie sind die Folge des Verbrauchs, nicht eines Rechenfehlers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wie sich der Verbrauch auf die Räume verteilt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heizkörper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einheiten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anteil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wohnzimmer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Wohnzimmer-Heizkörper allein macht über die Hälfte aus. Entweder läuft er dauerhaft, oder sein Bewertungsfaktor stimmt nicht.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Schlafzimmer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flur/Diele</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allgemeiner Raum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toilette</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Was zu prüfen ist, in dieser Reihenfolge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1  Techem-Abrechnung 2025 anfordern</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liegt noch nicht vor, wird aber für die Mieterabrechnung gebraucht. Dabei gleich die Bewertungsfaktoren der Heizkostenverteiler mit anfordern — die stehen nicht auf der Abrechnung, bestimmen aber, wie Ableseeinheiten in Kosten umgerechnet werden. Ein falsch parametrierter Heizkörper verzerrt alles.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2  Rohrwärme prüfen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der klassische Grund für Ausreißer nach oben: Laufen ungedämmte Heizungsleitungen sichtbar durch die Wohnung, geben sie Wärme ab, die die Heizkostenverteiler nicht messen — dafür heizen die Heizkörper mehr. § 7 Abs. 1 Satz 3 HeizkostenV erlaubt dann eine Korrektur nach VDI 2077. Bei einer Wohnung im Obergeschoss mit durchlaufenden Steigsträngen lohnt der Blick.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3  Wohnung ansehen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thermostatventile defekt oder dauerhaft offen? Fenster undicht? Dach gedämmt? Die Wohnung liegt im 2. Obergeschoss links, also oben — Wärmeverluste über die Decke sind dort am größten.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4  Mit dem Mieter sprechen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bei 208 % über dem Schnitt wird er eine Nachzahlung in dieser Höhe nicht kommentarlos zahlen. Besser vorher klären als hinterher streiten. Techem liefert seit 2022 monatliche Verbrauchsinformationen — er müsste den Verlauf kennen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5  Wirtschaftlich einordnen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Heizkosten trägt der Mieter, nicht du. Aber ein Verbrauch dieser Höhe drückt die erzielbare Kaltmiete und macht die Wohnung bei Neuvermietung schwer vermittelbar. Wenn eine Dämmung oder ein hydraulischer Abgleich das Dreifache auf das Übliche senkt, rechnet sich das über die Miete.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nebenbefund: CO₂-Kosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Liegenschaft stößt 25,3 kg CO₂ je Quadratmeter und Jahr aus. Nach dem CO₂-Kostenaufteilungsgesetz trägst du davon 30 Prozent — 2024 waren das 43,85 €. Techem weist den Betrag aus, zieht ihn aber nicht ab, weil die Verwaltung es so wollte. Du musst ihn dem Mieter erstatten; in der Abrechnung ist die Zeile dafür vorgesehen.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.00&quot; €&quot;;\-#,##0.00&quot; €&quot;;\-"/>
+    <numFmt numFmtId="166" formatCode="#,##0"/>
+    <numFmt numFmtId="167" formatCode="00\ %"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -450,7 +614,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="45">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -573,6 +737,62 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -827,7 +1047,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -1130,71 +1350,80 @@
       <c r="D33" s="15"/>
       <c r="E33" s="17"/>
     </row>
-    <row r="34" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="18" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34" s="15"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="17"/>
+    </row>
+    <row r="35" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B34" s="18"/>
-      <c r="C34" s="18"/>
-      <c r="D34" s="18"/>
-      <c r="E34" s="19" t="n">
-        <f aca="false">E33-E32</f>
+      <c r="B35" s="18"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="19" t="n">
+        <f aca="false">E33-E32+N(E34)</f>
         <v>-4527.84</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
-      <c r="D35" s="20"/>
-      <c r="E35" s="20"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B37" s="6"/>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6"/>
+      <c r="B36" s="20"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="20"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
+        <v>36</v>
+      </c>
       <c r="B38" s="6"/>
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
       <c r="E38" s="6"/>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="6"/>
+      <c r="B39" s="6"/>
+      <c r="C39" s="6"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="6"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="21"/>
-      <c r="B45" s="21"/>
-      <c r="C45" s="21"/>
-      <c r="D45" s="21"/>
-      <c r="E45" s="21"/>
-    </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="B46" s="20"/>
-      <c r="C46" s="20"/>
-      <c r="D46" s="20"/>
-      <c r="E46" s="20"/>
+      <c r="A46" s="21"/>
+      <c r="B46" s="21"/>
+      <c r="C46" s="21"/>
+      <c r="D46" s="21"/>
+      <c r="E46" s="21"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B47" s="20"/>
+      <c r="C47" s="20"/>
+      <c r="D47" s="20"/>
+      <c r="E47" s="20"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A11:E11"/>
@@ -1205,9 +1434,10 @@
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A33:D33"/>
     <mergeCell ref="A34:D34"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A37:E38"/>
-    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A38:E39"/>
+    <mergeCell ref="A47:E47"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1234,92 +1464,92 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="22" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="23" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="24" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="26"/>
       <c r="B5" s="27" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="24" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B7" s="25" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26"/>
       <c r="B8" s="27" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="29" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="30" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="29" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="30" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="29" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="30" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="29" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1331,4 +1561,313 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:E31"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="22" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="23" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="31"/>
+      <c r="B5" s="31" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="31" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" s="31" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="32" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" s="33" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="D6" s="34" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="32" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" s="33" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="33" t="s">
+        <v>68</v>
+      </c>
+      <c r="D7" s="34" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="C8" s="36" t="s">
+        <v>72</v>
+      </c>
+      <c r="D8" s="37" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="C9" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="D9" s="34" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="38" t="s">
+        <v>80</v>
+      </c>
+      <c r="B15" s="38" t="s">
+        <v>81</v>
+      </c>
+      <c r="C15" s="38" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" s="39" t="n">
+        <v>5794</v>
+      </c>
+      <c r="C16" s="40" t="n">
+        <f aca="false">B16/$B$22</f>
+        <v>0.535440347472507</v>
+      </c>
+      <c r="E16" s="41" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B17" s="39" t="n">
+        <v>2530</v>
+      </c>
+      <c r="C17" s="40" t="n">
+        <f aca="false">B17/$B$22</f>
+        <v>0.233804639127622</v>
+      </c>
+      <c r="E17" s="41"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B18" s="39" t="n">
+        <v>834</v>
+      </c>
+      <c r="C18" s="40" t="n">
+        <f aca="false">B18/$B$22</f>
+        <v>0.0770723593013585</v>
+      </c>
+      <c r="E18" s="41"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="B19" s="39" t="n">
+        <v>656</v>
+      </c>
+      <c r="C19" s="40" t="n">
+        <f aca="false">B19/$B$22</f>
+        <v>0.0606228629516681</v>
+      </c>
+      <c r="E19" s="41"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B20" s="39" t="n">
+        <v>682</v>
+      </c>
+      <c r="C20" s="40" t="n">
+        <f aca="false">B20/$B$22</f>
+        <v>0.0630255983735329</v>
+      </c>
+      <c r="E20" s="41"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" s="39" t="n">
+        <v>325</v>
+      </c>
+      <c r="C21" s="40" t="n">
+        <f aca="false">B21/$B$22</f>
+        <v>0.0300341927733112</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="B22" s="42" t="n">
+        <f aca="false">SUM(B16:B21)</f>
+        <v>10821</v>
+      </c>
+      <c r="C22" s="43"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+    </row>
+    <row r="26" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="44" t="s">
+        <v>94</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+    </row>
+    <row r="27" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="44" t="s">
+        <v>96</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+    </row>
+    <row r="28" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="44" t="s">
+        <v>98</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+    </row>
+    <row r="29" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="44" t="s">
+        <v>100</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+    </row>
+    <row r="31" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A11:E12"/>
+    <mergeCell ref="E16:E20"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B31:E31"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Mails zum Heizkostenthema Alzey, Zahlungshistorie bestaetigt
Drei Mailentwuerfe: an Steinmann Immobilien mit konkreten Forderungen und
Fachfragen zu Rohrwaerme und Geraetezustand, an Mazineler eine Vorwarnung
zur Nachzahlung mit Bitte um Ortstermin, und als zweiter Schritt eine an
Techem mit Fragen zu Bewertungsfaktoren, Geraetetausch und den monatlichen
Verbrauchsinformationen nach Paragraf 6a HeizkostenV.

Aus den Banking-Screenshots bestaetigt: Huber zahlte bis Mai 2026 je 890
EUR, ab Juni 2026 je 840 EUR - die Abrechnung 2025 steht damit endgueltig.
Mazineler zahlt durchgaengig 720 EUR; Aufteilung offen, zwei Eingaenge aus
2025 sind in der App rot markiert.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2Vxc1sWTkdQ9c9u5jSatw
</commit_message>
<xml_diff>
--- a/10_Output/2026-10-26-nebenkosten-2025-alzey-mazineler.xlsx
+++ b/10_Output/2026-10-26-nebenkosten-2025-alzey-mazineler.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Heizkosten pruefen" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Abrechnung!$A$1:$E$47</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Abrechnung!$A$1:$E$63</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">'Heizkosten pruefen'!$A$1:$E$32</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Hinweise und Fristen'!$A$1:$B$22</definedName>
   </definedNames>
@@ -88,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="116">
   <si>
     <t xml:space="preserve">Sascha Coldewey</t>
   </si>
@@ -205,6 +205,42 @@
   </si>
   <si>
     <t xml:space="preserve">Grundlage: Hausgeldabrechnung der Steinmann Immobilien für die WEG Langstraße 35+37 vom 18.06.2026, Einheit 0144.01.006.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Was bei welcher Aufteilung herauskommt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mazineler überweist seit mindestens 2025 durchgängig 720,00 € im Monat. Der Vertrag von 2021 nennt 600,00 €. Welcher Teil davon Vorauszahlung ist, steht nirgends — und genau das entscheidet über das Ergebnis:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annahme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaltmiete + Garage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vorauszahlung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">im Jahr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vorauszahlung unverändert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vorauszahlung auf 280 erhöht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vorauszahlung auf 320 erhöht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ein negatives Ergebnis ist die Nachzahlung, die auf Mazineler zukäme. Die mittlere Zeile entspricht am ehesten dem, was üblich wäre — aber geraten ist geraten. Nimm die Zahl aus dem Mietvertrag oder einer Erhöhungserklärung, falls es eine gibt, sonst aus einer Verständigung mit dem Mieter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Achtung: zwei Zahlungen 2025 auffällig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In der Banking-App sind die Eingänge vom 30.04.2025 und 30.05.2025 rot markiert. Falls das Rücklastschriften waren, hat Mazineler 2025 nicht zwölfmal gezahlt — dann ist die Summe der Vorauszahlungen entsprechend niedriger, und die offene Miete aus der Zahlungserinnerung vom März 2026 hat hier ihren Ursprung. Vor der Abrechnung im Kontoauszug nachsehen.</t>
   </si>
   <si>
     <t xml:space="preserve">Was du wissen musst</t>
@@ -499,17 +535,17 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b val="true"/>
       <sz val="9"/>
       <color rgb="FFC00000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="8">
@@ -614,7 +650,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="48">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -703,6 +739,26 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -711,15 +767,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -727,7 +779,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -777,10 +829,6 @@
     </xf>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1047,7 +1095,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -1422,8 +1470,148 @@
       <c r="D47" s="20"/>
       <c r="E47" s="20"/>
     </row>
+    <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B49" s="7"/>
+      <c r="C49" s="7"/>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+    </row>
+    <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B50" s="6"/>
+      <c r="C50" s="6"/>
+      <c r="D50" s="6"/>
+      <c r="E50" s="6"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="6"/>
+      <c r="B51" s="6"/>
+      <c r="C51" s="6"/>
+      <c r="D51" s="6"/>
+      <c r="E51" s="6"/>
+    </row>
+    <row r="53" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B53" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D53" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E53" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B54" s="12" t="n">
+        <v>520</v>
+      </c>
+      <c r="C54" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="D54" s="12" t="n">
+        <f aca="false">C54*12</f>
+        <v>2400</v>
+      </c>
+      <c r="E54" s="22" t="n">
+        <f aca="false">D54-$E$29</f>
+        <v>-2127.84</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B55" s="12" t="n">
+        <v>440</v>
+      </c>
+      <c r="C55" s="12" t="n">
+        <v>280</v>
+      </c>
+      <c r="D55" s="12" t="n">
+        <f aca="false">C55*12</f>
+        <v>3360</v>
+      </c>
+      <c r="E55" s="22" t="n">
+        <f aca="false">D55-$E$29</f>
+        <v>-1167.84</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B56" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="C56" s="12" t="n">
+        <v>320</v>
+      </c>
+      <c r="D56" s="12" t="n">
+        <f aca="false">C56*12</f>
+        <v>3840</v>
+      </c>
+      <c r="E56" s="22" t="n">
+        <f aca="false">D56-$E$29</f>
+        <v>-687.84</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="B57" s="23"/>
+      <c r="C57" s="23"/>
+      <c r="D57" s="23"/>
+      <c r="E57" s="23"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="23"/>
+      <c r="B58" s="23"/>
+      <c r="C58" s="23"/>
+      <c r="D58" s="23"/>
+      <c r="E58" s="23"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="B60" s="25"/>
+      <c r="C60" s="25"/>
+      <c r="D60" s="25"/>
+      <c r="E60" s="25"/>
+    </row>
+    <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="B61" s="26"/>
+      <c r="C61" s="26"/>
+      <c r="D61" s="26"/>
+      <c r="E61" s="26"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="26"/>
+      <c r="B62" s="26"/>
+      <c r="C62" s="26"/>
+      <c r="D62" s="26"/>
+      <c r="E62" s="26"/>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="18">
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A11:E11"/>
@@ -1438,6 +1626,10 @@
     <mergeCell ref="A36:E36"/>
     <mergeCell ref="A38:E39"/>
     <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A50:E51"/>
+    <mergeCell ref="A57:E58"/>
+    <mergeCell ref="A61:E62"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1463,93 +1655,93 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="22" t="s">
-        <v>39</v>
+      <c r="A1" s="27" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="23" t="s">
-        <v>40</v>
+      <c r="A2" s="28" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="B4" s="25" t="s">
-        <v>42</v>
+      <c r="A4" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="26"/>
-      <c r="B5" s="27" t="s">
-        <v>43</v>
+      <c r="A5" s="25"/>
+      <c r="B5" s="31" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="B7" s="25" t="s">
-        <v>44</v>
+      <c r="A7" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="26"/>
-      <c r="B8" s="27" t="s">
-        <v>45</v>
+      <c r="A8" s="25"/>
+      <c r="B8" s="31" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="28" t="s">
-        <v>46</v>
+      <c r="A10" s="32" t="s">
+        <v>58</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="29" t="s">
-        <v>48</v>
+      <c r="B11" s="33" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="30" t="s">
-        <v>49</v>
+      <c r="A13" s="34" t="s">
+        <v>61</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="29" t="s">
-        <v>51</v>
+      <c r="B14" s="33" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="30" t="s">
-        <v>49</v>
+      <c r="A16" s="34" t="s">
+        <v>61</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="29" t="s">
-        <v>53</v>
+      <c r="B17" s="33" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="30" t="s">
-        <v>49</v>
+      <c r="A19" s="34" t="s">
+        <v>61</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="29" t="s">
-        <v>55</v>
+      <c r="B20" s="33" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1577,91 +1769,91 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="22" t="s">
-        <v>56</v>
+      <c r="A1" s="27" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="23" t="s">
-        <v>57</v>
+      <c r="A2" s="28" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="31"/>
-      <c r="B5" s="31" t="s">
-        <v>59</v>
-      </c>
-      <c r="C5" s="31" t="s">
-        <v>60</v>
-      </c>
-      <c r="D5" s="31" t="s">
-        <v>61</v>
+      <c r="A5" s="35"/>
+      <c r="B5" s="35" t="s">
+        <v>71</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" s="35" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="32" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" s="33" t="s">
-        <v>63</v>
-      </c>
-      <c r="C6" s="33" t="s">
-        <v>64</v>
-      </c>
-      <c r="D6" s="34" t="s">
-        <v>65</v>
+      <c r="A6" s="36" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" s="37" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6" s="37" t="s">
+        <v>76</v>
+      </c>
+      <c r="D6" s="38" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="32" t="s">
-        <v>66</v>
-      </c>
-      <c r="B7" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="C7" s="33" t="s">
-        <v>68</v>
-      </c>
-      <c r="D7" s="34" t="s">
-        <v>69</v>
+      <c r="A7" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="37" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="38" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="35" t="s">
-        <v>70</v>
-      </c>
-      <c r="B8" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="C8" s="36" t="s">
-        <v>72</v>
-      </c>
-      <c r="D8" s="37" t="s">
-        <v>73</v>
+      <c r="A8" s="39" t="s">
+        <v>82</v>
+      </c>
+      <c r="B8" s="40" t="s">
+        <v>83</v>
+      </c>
+      <c r="C8" s="40" t="s">
+        <v>84</v>
+      </c>
+      <c r="D8" s="41" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="32" t="s">
-        <v>74</v>
-      </c>
-      <c r="B9" s="33" t="s">
-        <v>75</v>
-      </c>
-      <c r="C9" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="D9" s="34" t="s">
-        <v>77</v>
+      <c r="A9" s="36" t="s">
+        <v>86</v>
+      </c>
+      <c r="B9" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="C9" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="D9" s="38" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -1677,164 +1869,164 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="38" t="s">
-        <v>80</v>
-      </c>
-      <c r="B15" s="38" t="s">
-        <v>81</v>
-      </c>
-      <c r="C15" s="38" t="s">
-        <v>82</v>
+      <c r="A15" s="42" t="s">
+        <v>92</v>
+      </c>
+      <c r="B15" s="42" t="s">
+        <v>93</v>
+      </c>
+      <c r="C15" s="42" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="B16" s="39" t="n">
+        <v>95</v>
+      </c>
+      <c r="B16" s="43" t="n">
         <v>5794</v>
       </c>
-      <c r="C16" s="40" t="n">
+      <c r="C16" s="44" t="n">
         <f aca="false">B16/$B$22</f>
         <v>0.535440347472507</v>
       </c>
-      <c r="E16" s="41" t="s">
-        <v>84</v>
+      <c r="E16" s="23" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="B17" s="39" t="n">
+        <v>97</v>
+      </c>
+      <c r="B17" s="43" t="n">
         <v>2530</v>
       </c>
-      <c r="C17" s="40" t="n">
+      <c r="C17" s="44" t="n">
         <f aca="false">B17/$B$22</f>
         <v>0.233804639127622</v>
       </c>
-      <c r="E17" s="41"/>
+      <c r="E17" s="23"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="B18" s="39" t="n">
+        <v>98</v>
+      </c>
+      <c r="B18" s="43" t="n">
         <v>834</v>
       </c>
-      <c r="C18" s="40" t="n">
+      <c r="C18" s="44" t="n">
         <f aca="false">B18/$B$22</f>
         <v>0.0770723593013585</v>
       </c>
-      <c r="E18" s="41"/>
+      <c r="E18" s="23"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="B19" s="39" t="n">
+        <v>99</v>
+      </c>
+      <c r="B19" s="43" t="n">
         <v>656</v>
       </c>
-      <c r="C19" s="40" t="n">
+      <c r="C19" s="44" t="n">
         <f aca="false">B19/$B$22</f>
         <v>0.0606228629516681</v>
       </c>
-      <c r="E19" s="41"/>
+      <c r="E19" s="23"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="B20" s="39" t="n">
+        <v>100</v>
+      </c>
+      <c r="B20" s="43" t="n">
         <v>682</v>
       </c>
-      <c r="C20" s="40" t="n">
+      <c r="C20" s="44" t="n">
         <f aca="false">B20/$B$22</f>
         <v>0.0630255983735329</v>
       </c>
-      <c r="E20" s="41"/>
+      <c r="E20" s="23"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="B21" s="39" t="n">
+        <v>101</v>
+      </c>
+      <c r="B21" s="43" t="n">
         <v>325</v>
       </c>
-      <c r="C21" s="40" t="n">
+      <c r="C21" s="44" t="n">
         <f aca="false">B21/$B$22</f>
         <v>0.0300341927733112</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="B22" s="42" t="n">
+        <v>102</v>
+      </c>
+      <c r="B22" s="45" t="n">
         <f aca="false">SUM(B16:B21)</f>
         <v>10821</v>
       </c>
-      <c r="C22" s="43"/>
+      <c r="C22" s="46"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="44" t="s">
-        <v>92</v>
+      <c r="A25" s="47" t="s">
+        <v>104</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
     </row>
     <row r="26" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="44" t="s">
-        <v>94</v>
+      <c r="A26" s="47" t="s">
+        <v>106</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
       <c r="E26" s="6"/>
     </row>
     <row r="27" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="44" t="s">
-        <v>96</v>
+      <c r="A27" s="47" t="s">
+        <v>108</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
       <c r="E27" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="44" t="s">
-        <v>98</v>
+      <c r="A28" s="47" t="s">
+        <v>110</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
       <c r="E28" s="6"/>
     </row>
     <row r="29" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="44" t="s">
-        <v>100</v>
+      <c r="A29" s="47" t="s">
+        <v>112</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
@@ -1842,10 +2034,10 @@
     </row>
     <row r="31" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>

</xml_diff>

<commit_message>
Standbericht als PDF, offene Miete Alzey, Niessbrauch geloescht
Fuenfseitiger Standbericht beider Wohnungen nach War, Ist, Soll mit
Kennzahlenvergleich und Priorisierung.

Alzey: Die Eingaenge vom 30.04. und 30.05.2025 wurden zurueckgebucht, unterm
Strich fehlt die Miete Mai 2025 ueber 720 EUR. Schreiben dazu erstellt. Die
Abrechnung rechnet jetzt mit elf statt zwoelf Monaten Vorauszahlung; je nach
Aufteilung ergibt sich eine Nachzahlung zwischen 1.008 und 2.328 EUR.
Zusammen mit der offenen Miete kommen 1.720 bis 3.050 EUR auf den Mieter zu.

Der Niessbrauch ist abgeloest und im Grundbuch geloescht, die Wohnung damit
lastenfrei.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2Vxc1sWTkdQ9c9u5jSatw
</commit_message>
<xml_diff>
--- a/10_Output/2026-10-26-nebenkosten-2025-alzey-mazineler.xlsx
+++ b/10_Output/2026-10-26-nebenkosten-2025-alzey-mazineler.xlsx
@@ -65,8 +65,8 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">FEHLT: Summe der 2025 tatsächlich gezahlten Vorauszahlungen eintragen.
-Laut Mietvertrag von 2021 wären es 200 € im Monat, also 2.400 €. Tatsächlich überweist Mazineler aber 720 € brutto statt der vertraglichen 600 € — die Aufteilung ist ungeklärt.
-Danach rechnet sich das Ergebnis von selbst.</t>
+Achtung: Die Miete Mai 2025 wurde nie gezahlt, die Lastschrift ging zurück. Es sind also elf Monate, nicht zwölf.
+Wie sich die 720 € in Kaltmiete, Garage und Vorauszahlung aufteilen, ist ungeklärt — siehe die Szenarien weiter unten.</t>
         </r>
       </text>
     </comment>
@@ -222,7 +222,7 @@
     <t xml:space="preserve">Vorauszahlung</t>
   </si>
   <si>
-    <t xml:space="preserve">im Jahr</t>
+    <t xml:space="preserve">11 Monate</t>
   </si>
   <si>
     <t xml:space="preserve">Vorauszahlung unverändert</t>
@@ -237,10 +237,11 @@
     <t xml:space="preserve">Ein negatives Ergebnis ist die Nachzahlung, die auf Mazineler zukäme. Die mittlere Zeile entspricht am ehesten dem, was üblich wäre — aber geraten ist geraten. Nimm die Zahl aus dem Mietvertrag oder einer Erhöhungserklärung, falls es eine gibt, sonst aus einer Verständigung mit dem Mieter.</t>
   </si>
   <si>
-    <t xml:space="preserve">Achtung: zwei Zahlungen 2025 auffällig</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In der Banking-App sind die Eingänge vom 30.04.2025 und 30.05.2025 rot markiert. Falls das Rücklastschriften waren, hat Mazineler 2025 nicht zwölfmal gezahlt — dann ist die Summe der Vorauszahlungen entsprechend niedriger, und die offene Miete aus der Zahlungserinnerung vom März 2026 hat hier ihren Ursprung. Vor der Abrechnung im Kontoauszug nachsehen.</t>
+    <t xml:space="preserve">Die Miete Mai 2025 ist offen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Lastschrift wurde zurückgegeben, gezahlt wurde nie. Deshalb rechnen die Spalten oben mit elf statt zwölf Monaten — die in der Maimiete enthaltene Vorauszahlung ist nie geflossen und darf nicht angerechnet werden.
+Die offene Miete selbst gehört nicht in diese Abrechnung: Sie ist eine eigene Forderung über 720,00 € und wird getrennt geltend gemacht. Verjährung tritt erst Ende 2028 ein, Eile besteht also nicht — aber liegen lassen sollte man sie auch nicht.</t>
   </si>
   <si>
     <t xml:space="preserve">Was du wissen musst</t>
@@ -1523,12 +1524,12 @@
         <v>200</v>
       </c>
       <c r="D54" s="12" t="n">
-        <f aca="false">C54*12</f>
-        <v>2400</v>
+        <f aca="false">C54*11</f>
+        <v>2200</v>
       </c>
       <c r="E54" s="22" t="n">
         <f aca="false">D54-$E$29</f>
-        <v>-2127.84</v>
+        <v>-2327.84</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1542,12 +1543,12 @@
         <v>280</v>
       </c>
       <c r="D55" s="12" t="n">
-        <f aca="false">C55*12</f>
-        <v>3360</v>
+        <f aca="false">C55*11</f>
+        <v>3080</v>
       </c>
       <c r="E55" s="22" t="n">
         <f aca="false">D55-$E$29</f>
-        <v>-1167.84</v>
+        <v>-1447.84</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1561,12 +1562,12 @@
         <v>320</v>
       </c>
       <c r="D56" s="12" t="n">
-        <f aca="false">C56*12</f>
-        <v>3840</v>
+        <f aca="false">C56*11</f>
+        <v>3520</v>
       </c>
       <c r="E56" s="22" t="n">
         <f aca="false">D56-$E$29</f>
-        <v>-687.84</v>
+        <v>-1007.84</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>